<commit_message>
alteração do BS_ERROR para 0.91 cm, para correção sistemática do erro de medição do Kinect Orbbec.
</commit_message>
<xml_diff>
--- a/arquivos/tabelas_testes/sit_and_reach_test_orbbec.xlsx
+++ b/arquivos/tabelas_testes/sit_and_reach_test_orbbec.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -561,20 +561,14 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
+      <c r="A5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B5" t="n">
+        <v>165</v>
+      </c>
+      <c r="C5" t="n">
+        <v>63</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -594,6 +588,72 @@
       </c>
       <c r="H5" t="n">
         <v>1.93</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B6" t="n">
+        <v>165</v>
+      </c>
+      <c r="C6" t="n">
+        <v>63</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-1.32</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.32</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-3.13</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3.13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
alteração de salvamento de dados e correção de flip de imagem que não existia na orbbec
</commit_message>
<xml_diff>
--- a/arquivos/tabelas_testes/sit_and_reach_test_orbbec.xlsx
+++ b/arquivos/tabelas_testes/sit_and_reach_test_orbbec.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1701,20 +1701,14 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
+      <c r="A43" t="n">
+        <v>22</v>
+      </c>
+      <c r="B43" t="n">
+        <v>165</v>
+      </c>
+      <c r="C43" t="n">
+        <v>63</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1734,6 +1728,42 @@
       </c>
       <c r="H43" t="n">
         <v>0.74</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>